<commit_message>
redid the code and did report v3 and v4
</commit_message>
<xml_diff>
--- a/data/comments/eval_report_coding_v3.xlsx
+++ b/data/comments/eval_report_coding_v3.xlsx
@@ -505,25 +505,25 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.9642857142857143</v>
+        <v>0.9586776859504132</v>
       </c>
       <c r="F2" t="n">
-        <v>0.907563025210084</v>
+        <v>0.9747899159663865</v>
       </c>
       <c r="G2" t="n">
-        <v>0.935064935064935</v>
+        <v>0.9666666666666667</v>
       </c>
       <c r="H2" t="n">
         <v>119</v>
       </c>
       <c r="I2" t="n">
-        <v>0.889</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>0.553</v>
+        <v>0.7</v>
       </c>
       <c r="K2" t="n">
-        <v>0.552</v>
+        <v>0.701</v>
       </c>
     </row>
     <row r="3">
@@ -546,25 +546,25 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.5217391304347826</v>
+        <v>0.7857142857142857</v>
       </c>
       <c r="F3" t="n">
-        <v>0.75</v>
+        <v>0.6875</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6153846153846154</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="H3" t="n">
         <v>16</v>
       </c>
       <c r="I3" t="n">
-        <v>0.889</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>0.553</v>
+        <v>0.7</v>
       </c>
       <c r="K3" t="n">
-        <v>0.552</v>
+        <v>0.701</v>
       </c>
     </row>
     <row r="4">
@@ -587,25 +587,25 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.7430124223602484</v>
+        <v>0.8721959858323495</v>
       </c>
       <c r="F4" t="n">
-        <v>0.828781512605042</v>
+        <v>0.8311449579831933</v>
       </c>
       <c r="G4" t="n">
-        <v>0.7752247752247752</v>
+        <v>0.85</v>
       </c>
       <c r="H4" t="n">
         <v>135</v>
       </c>
       <c r="I4" t="n">
-        <v>0.889</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>0.553</v>
+        <v>0.7</v>
       </c>
       <c r="K4" t="n">
-        <v>0.552</v>
+        <v>0.701</v>
       </c>
     </row>
     <row r="5">
@@ -628,25 +628,25 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.9118357487922705</v>
+        <v>0.9381783199965018</v>
       </c>
       <c r="F5" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.9407407407407408</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8971768971768972</v>
+        <v>0.9390123456790124</v>
       </c>
       <c r="H5" t="n">
         <v>135</v>
       </c>
       <c r="I5" t="n">
-        <v>0.889</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>0.553</v>
+        <v>0.7</v>
       </c>
       <c r="K5" t="n">
-        <v>0.552</v>
+        <v>0.701</v>
       </c>
     </row>
     <row r="6">
@@ -669,25 +669,25 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.9705882352941176</v>
+        <v>0.8924731182795699</v>
       </c>
       <c r="F6" t="n">
-        <v>0.33</v>
+        <v>0.83</v>
       </c>
       <c r="G6" t="n">
-        <v>0.4925373134328358</v>
+        <v>0.8601036269430051</v>
       </c>
       <c r="H6" t="n">
         <v>100</v>
       </c>
       <c r="I6" t="n">
-        <v>0.496</v>
+        <v>0.8</v>
       </c>
       <c r="J6" t="n">
-        <v>0.187</v>
+        <v>0.511</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.004</v>
+        <v>0.511</v>
       </c>
     </row>
     <row r="7">
@@ -710,25 +710,25 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.3366336633663367</v>
+        <v>0.5952380952380952</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9714285714285714</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5</v>
+        <v>0.6493506493506493</v>
       </c>
       <c r="H7" t="n">
         <v>35</v>
       </c>
       <c r="I7" t="n">
-        <v>0.496</v>
+        <v>0.8</v>
       </c>
       <c r="J7" t="n">
-        <v>0.187</v>
+        <v>0.511</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.004</v>
+        <v>0.511</v>
       </c>
     </row>
     <row r="8">
@@ -751,25 +751,25 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.6536109493302271</v>
+        <v>0.7438556067588326</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6507142857142857</v>
+        <v>0.7721428571428571</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4962686567164179</v>
+        <v>0.7547271381468272</v>
       </c>
       <c r="H8" t="n">
         <v>135</v>
       </c>
       <c r="I8" t="n">
-        <v>0.496</v>
+        <v>0.8</v>
       </c>
       <c r="J8" t="n">
-        <v>0.187</v>
+        <v>0.511</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.004</v>
+        <v>0.511</v>
       </c>
     </row>
     <row r="9">
@@ -792,25 +792,25 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.8062296425721004</v>
+        <v>0.8154121863799283</v>
       </c>
       <c r="F9" t="n">
-        <v>0.4962962962962963</v>
+        <v>0.8</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4944720840243229</v>
+        <v>0.8054639660857277</v>
       </c>
       <c r="H9" t="n">
         <v>135</v>
       </c>
       <c r="I9" t="n">
-        <v>0.496</v>
+        <v>0.8</v>
       </c>
       <c r="J9" t="n">
-        <v>0.187</v>
+        <v>0.511</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.004</v>
+        <v>0.511</v>
       </c>
     </row>
     <row r="10">
@@ -833,25 +833,25 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0.7425742574257426</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.974025974025974</v>
       </c>
       <c r="G10" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.8426966292134831</v>
       </c>
       <c r="H10" t="n">
         <v>77</v>
       </c>
       <c r="I10" t="n">
-        <v>0.593</v>
+        <v>0.793</v>
       </c>
       <c r="J10" t="n">
-        <v>0.256</v>
+        <v>0.554</v>
       </c>
       <c r="K10" t="n">
-        <v>0.126</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="11">
@@ -874,25 +874,25 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.5132743362831859</v>
+        <v>0.9411764705882353</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0.5517241379310345</v>
       </c>
       <c r="G11" t="n">
-        <v>0.6783625730994152</v>
+        <v>0.6956521739130435</v>
       </c>
       <c r="H11" t="n">
         <v>58</v>
       </c>
       <c r="I11" t="n">
-        <v>0.593</v>
+        <v>0.793</v>
       </c>
       <c r="J11" t="n">
-        <v>0.256</v>
+        <v>0.554</v>
       </c>
       <c r="K11" t="n">
-        <v>0.126</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="12">
@@ -915,25 +915,25 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.7566371681415929</v>
+        <v>0.8418753640069889</v>
       </c>
       <c r="F12" t="n">
-        <v>0.6428571428571428</v>
+        <v>0.7628750559785042</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5614035087719298</v>
+        <v>0.7691744015632633</v>
       </c>
       <c r="H12" t="n">
         <v>135</v>
       </c>
       <c r="I12" t="n">
-        <v>0.593</v>
+        <v>0.793</v>
       </c>
       <c r="J12" t="n">
-        <v>0.256</v>
+        <v>0.554</v>
       </c>
       <c r="K12" t="n">
-        <v>0.126</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="13">
@@ -956,25 +956,25 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.7908882333661095</v>
+        <v>0.827899652710369</v>
       </c>
       <c r="F13" t="n">
-        <v>0.5925925925925926</v>
+        <v>0.7925925925925926</v>
       </c>
       <c r="G13" t="n">
-        <v>0.5449426034221355</v>
+        <v>0.7795219743436645</v>
       </c>
       <c r="H13" t="n">
         <v>135</v>
       </c>
       <c r="I13" t="n">
-        <v>0.593</v>
+        <v>0.793</v>
       </c>
       <c r="J13" t="n">
-        <v>0.256</v>
+        <v>0.554</v>
       </c>
       <c r="K13" t="n">
-        <v>0.126</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="14">
@@ -997,25 +997,25 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>0.59375</v>
       </c>
       <c r="F14" t="n">
-        <v>0.103448275862069</v>
+        <v>0.6551724137931034</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1875</v>
+        <v>0.6229508196721312</v>
       </c>
       <c r="H14" t="n">
         <v>29</v>
       </c>
       <c r="I14" t="n">
-        <v>0.533</v>
+        <v>0.526</v>
       </c>
       <c r="J14" t="n">
-        <v>0.536</v>
+        <v>0.58</v>
       </c>
       <c r="K14" t="n">
-        <v>0.667</v>
+        <v>0.759</v>
       </c>
     </row>
     <row r="15">
@@ -1038,25 +1038,25 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4222222222222222</v>
+        <v>0.38</v>
       </c>
       <c r="F15" t="n">
         <v>0.475</v>
       </c>
       <c r="G15" t="n">
-        <v>0.4470588235294118</v>
+        <v>0.4222222222222222</v>
       </c>
       <c r="H15" t="n">
         <v>40</v>
       </c>
       <c r="I15" t="n">
-        <v>0.533</v>
+        <v>0.526</v>
       </c>
       <c r="J15" t="n">
-        <v>0.536</v>
+        <v>0.58</v>
       </c>
       <c r="K15" t="n">
-        <v>0.667</v>
+        <v>0.759</v>
       </c>
     </row>
     <row r="16">
@@ -1079,25 +1079,25 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.4772727272727273</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="F16" t="n">
-        <v>0.6</v>
+        <v>0.3428571428571429</v>
       </c>
       <c r="G16" t="n">
-        <v>0.5316455696202531</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="H16" t="n">
         <v>35</v>
       </c>
       <c r="I16" t="n">
-        <v>0.533</v>
+        <v>0.526</v>
       </c>
       <c r="J16" t="n">
-        <v>0.536</v>
+        <v>0.58</v>
       </c>
       <c r="K16" t="n">
-        <v>0.667</v>
+        <v>0.759</v>
       </c>
     </row>
     <row r="17">
@@ -1120,25 +1120,25 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.6744186046511628</v>
+        <v>0.8076923076923077</v>
       </c>
       <c r="F17" t="n">
-        <v>0.9354838709677419</v>
+        <v>0.6774193548387096</v>
       </c>
       <c r="G17" t="n">
-        <v>0.7837837837837838</v>
+        <v>0.7368421052631579</v>
       </c>
       <c r="H17" t="n">
         <v>31</v>
       </c>
       <c r="I17" t="n">
-        <v>0.533</v>
+        <v>0.526</v>
       </c>
       <c r="J17" t="n">
-        <v>0.536</v>
+        <v>0.58</v>
       </c>
       <c r="K17" t="n">
-        <v>0.667</v>
+        <v>0.759</v>
       </c>
     </row>
     <row r="18">
@@ -1161,25 +1161,25 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.6434783885365281</v>
+        <v>0.556471688034188</v>
       </c>
       <c r="F18" t="n">
-        <v>0.5284830367074527</v>
+        <v>0.5376122278722389</v>
       </c>
       <c r="G18" t="n">
-        <v>0.4874970442333622</v>
+        <v>0.542277980337765</v>
       </c>
       <c r="H18" t="n">
         <v>135</v>
       </c>
       <c r="I18" t="n">
-        <v>0.533</v>
+        <v>0.526</v>
       </c>
       <c r="J18" t="n">
-        <v>0.536</v>
+        <v>0.58</v>
       </c>
       <c r="K18" t="n">
-        <v>0.667</v>
+        <v>0.759</v>
       </c>
     </row>
     <row r="19">
@@ -1202,25 +1202,25 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.6185215636120029</v>
+        <v>0.5408353118075341</v>
       </c>
       <c r="F19" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5259259259259259</v>
       </c>
       <c r="G19" t="n">
-        <v>0.4905536679643157</v>
+        <v>0.5284811482912057</v>
       </c>
       <c r="H19" t="n">
         <v>135</v>
       </c>
       <c r="I19" t="n">
-        <v>0.533</v>
+        <v>0.526</v>
       </c>
       <c r="J19" t="n">
-        <v>0.536</v>
+        <v>0.58</v>
       </c>
       <c r="K19" t="n">
-        <v>0.667</v>
+        <v>0.759</v>
       </c>
     </row>
     <row r="20">
@@ -1246,22 +1246,22 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>0.5</v>
+        <v>0.125</v>
       </c>
       <c r="G20" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="H20" t="n">
         <v>16</v>
       </c>
       <c r="I20" t="n">
-        <v>0.533</v>
+        <v>0.526</v>
       </c>
       <c r="J20" t="n">
-        <v>0.184</v>
+        <v>0.196</v>
       </c>
       <c r="K20" t="n">
-        <v>0.081</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="21">
@@ -1284,25 +1284,25 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.5166666666666667</v>
+        <v>0.5535714285714286</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>0.6813186813186813</v>
+        <v>0.7126436781609196</v>
       </c>
       <c r="H21" t="n">
         <v>62</v>
       </c>
       <c r="I21" t="n">
-        <v>0.533</v>
+        <v>0.526</v>
       </c>
       <c r="J21" t="n">
-        <v>0.184</v>
+        <v>0.196</v>
       </c>
       <c r="K21" t="n">
-        <v>0.081</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="22">
@@ -1325,25 +1325,25 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.4</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F22" t="n">
         <v>0.05128205128205128</v>
       </c>
       <c r="G22" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.08888888888888889</v>
       </c>
       <c r="H22" t="n">
         <v>39</v>
       </c>
       <c r="I22" t="n">
-        <v>0.533</v>
+        <v>0.526</v>
       </c>
       <c r="J22" t="n">
-        <v>0.184</v>
+        <v>0.196</v>
       </c>
       <c r="K22" t="n">
-        <v>0.081</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="23">
@@ -1366,25 +1366,25 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>0.2777777777777778</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="H23" t="n">
         <v>18</v>
       </c>
       <c r="I23" t="n">
-        <v>0.533</v>
+        <v>0.526</v>
       </c>
       <c r="J23" t="n">
-        <v>0.184</v>
+        <v>0.196</v>
       </c>
       <c r="K23" t="n">
-        <v>0.081</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="24">
@@ -1407,25 +1407,25 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.4791666666666666</v>
+        <v>0.5550595238095238</v>
       </c>
       <c r="F24" t="n">
-        <v>0.3878205128205128</v>
+        <v>0.3635149572649573</v>
       </c>
       <c r="G24" t="n">
-        <v>0.3597236097236097</v>
+        <v>0.3316962730755834</v>
       </c>
       <c r="H24" t="n">
         <v>135</v>
       </c>
       <c r="I24" t="n">
-        <v>0.533</v>
+        <v>0.526</v>
       </c>
       <c r="J24" t="n">
-        <v>0.184</v>
+        <v>0.196</v>
       </c>
       <c r="K24" t="n">
-        <v>0.081</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="25">
@@ -1448,25 +1448,25 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.4713580246913581</v>
+        <v>0.5134920634920636</v>
       </c>
       <c r="F25" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5259259259259259</v>
       </c>
       <c r="G25" t="n">
-        <v>0.4181768848435515</v>
+        <v>0.4197087090573681</v>
       </c>
       <c r="H25" t="n">
         <v>135</v>
       </c>
       <c r="I25" t="n">
-        <v>0.533</v>
+        <v>0.526</v>
       </c>
       <c r="J25" t="n">
-        <v>0.184</v>
+        <v>0.196</v>
       </c>
       <c r="K25" t="n">
-        <v>0.081</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="26">
@@ -1489,25 +1489,25 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.8526315789473684</v>
       </c>
       <c r="F26" t="n">
-        <v>0.5842696629213483</v>
+        <v>0.9101123595505618</v>
       </c>
       <c r="G26" t="n">
-        <v>0.7172413793103448</v>
+        <v>0.8804347826086957</v>
       </c>
       <c r="H26" t="n">
         <v>89</v>
       </c>
       <c r="I26" t="n">
-        <v>0.696</v>
+        <v>0.837</v>
       </c>
       <c r="J26" t="n">
-        <v>0.424</v>
+        <v>0.625</v>
       </c>
       <c r="K26" t="n">
-        <v>0.392</v>
+        <v>0.626</v>
       </c>
     </row>
     <row r="27">
@@ -1530,25 +1530,25 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.5316455696202531</v>
+        <v>0.8</v>
       </c>
       <c r="F27" t="n">
-        <v>0.9130434782608695</v>
+        <v>0.6956521739130435</v>
       </c>
       <c r="G27" t="n">
-        <v>0.672</v>
+        <v>0.7441860465116279</v>
       </c>
       <c r="H27" t="n">
         <v>46</v>
       </c>
       <c r="I27" t="n">
-        <v>0.696</v>
+        <v>0.837</v>
       </c>
       <c r="J27" t="n">
-        <v>0.424</v>
+        <v>0.625</v>
       </c>
       <c r="K27" t="n">
-        <v>0.392</v>
+        <v>0.626</v>
       </c>
     </row>
     <row r="28">
@@ -1571,25 +1571,25 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.7301084990958409</v>
+        <v>0.8263157894736842</v>
       </c>
       <c r="F28" t="n">
-        <v>0.7486565705911089</v>
+        <v>0.8028822667318026</v>
       </c>
       <c r="G28" t="n">
-        <v>0.6946206896551724</v>
+        <v>0.8123104145601618</v>
       </c>
       <c r="H28" t="n">
         <v>135</v>
       </c>
       <c r="I28" t="n">
-        <v>0.696</v>
+        <v>0.837</v>
       </c>
       <c r="J28" t="n">
-        <v>0.424</v>
+        <v>0.625</v>
       </c>
       <c r="K28" t="n">
-        <v>0.392</v>
+        <v>0.626</v>
       </c>
     </row>
     <row r="29">
@@ -1612,25 +1612,25 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.7933226173732503</v>
+        <v>0.8346978557504873</v>
       </c>
       <c r="F29" t="n">
-        <v>0.6962962962962963</v>
+        <v>0.837037037037037</v>
       </c>
       <c r="G29" t="n">
-        <v>0.7018257982120051</v>
+        <v>0.8340092873459911</v>
       </c>
       <c r="H29" t="n">
         <v>135</v>
       </c>
       <c r="I29" t="n">
-        <v>0.696</v>
+        <v>0.837</v>
       </c>
       <c r="J29" t="n">
-        <v>0.424</v>
+        <v>0.625</v>
       </c>
       <c r="K29" t="n">
-        <v>0.392</v>
+        <v>0.626</v>
       </c>
     </row>
   </sheetData>

</xml_diff>